<commit_message>
baseyear update 11th Oct
1st version of base year update(11th Oct)
</commit_message>
<xml_diff>
--- a/input/gcamdata/inst/extdata/gcam-china/key results_comparison_all_years.xlsx
+++ b/input/gcamdata/inst/extdata/gcam-china/key results_comparison_all_years.xlsx
@@ -1,32 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yarl762\Desktop\GitHub\gcamdata\inst\extdata\gcam-china\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62A2DE42-409A-4710-B51E-E8B8BC9A6A47}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="2445" yWindow="2025" windowWidth="25545" windowHeight="11925" xr2:uid="{0B294428-86F4-427F-A0C2-2C1D608EAB2D}"/>
+    <workbookView windowWidth="22395" windowHeight="11670"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
@@ -42,7 +25,28 @@
     <t>Unit</t>
   </si>
   <si>
+    <t>1.5C Core</t>
+  </si>
+  <si>
+    <t xml:space="preserve">global GHG </t>
+  </si>
+  <si>
+    <t>MtCO2e</t>
+  </si>
+  <si>
+    <t>China GHG</t>
+  </si>
+  <si>
+    <t>global net CO2</t>
+  </si>
+  <si>
+    <t>MtCO2</t>
+  </si>
+  <si>
     <t>global energy CO2</t>
+  </si>
+  <si>
+    <t>China net CO2</t>
   </si>
   <si>
     <t>China energy CO2</t>
@@ -51,79 +55,401 @@
     <t>China total elec gen</t>
   </si>
   <si>
+    <t>TWh</t>
+  </si>
+  <si>
     <t>China elec gen by coal</t>
   </si>
   <si>
     <t>temperature</t>
   </si>
   <si>
-    <t>1.5C Core</t>
+    <t>degC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">climate forcing </t>
+  </si>
+  <si>
+    <t>W/m^2</t>
+  </si>
+  <si>
+    <t>CO2 prices</t>
+  </si>
+  <si>
+    <t>2017$/tCO2</t>
   </si>
   <si>
     <t>2C Core</t>
   </si>
   <si>
-    <t xml:space="preserve">global GHG </t>
-  </si>
-  <si>
-    <t>China GHG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">climate forcing </t>
-  </si>
-  <si>
-    <t>CO2 prices</t>
-  </si>
-  <si>
-    <t>global net CO2</t>
-  </si>
-  <si>
-    <t>China net CO2</t>
-  </si>
-  <si>
     <t>REF</t>
-  </si>
-  <si>
-    <t>MtCO2e</t>
-  </si>
-  <si>
-    <t>MtCO2</t>
-  </si>
-  <si>
-    <t>TWh</t>
-  </si>
-  <si>
-    <t>degC</t>
-  </si>
-  <si>
-    <t>W/m^2</t>
-  </si>
-  <si>
-    <t>2017$/tCO2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="等线"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -131,25 +457,311 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -198,7 +810,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -231,26 +843,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -283,23 +878,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -441,27 +1019,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{776DB30E-CCD5-4724-B9B5-D6B90C23A2FB}">
-  <dimension ref="A1:W34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:X34"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="20" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.7083333333333" customWidth="1"/>
+    <col min="3" max="21" width="9.28333333333333" customWidth="1"/>
+    <col min="22" max="22" width="11" customWidth="1"/>
+    <col min="23" max="23" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -481,137 +1054,143 @@
         <v>2020</v>
       </c>
       <c r="G1">
+        <v>2021</v>
+      </c>
+      <c r="H1">
         <v>2025</v>
       </c>
-      <c r="H1">
+      <c r="I1">
         <v>2030</v>
       </c>
-      <c r="I1">
+      <c r="J1">
         <v>2035</v>
       </c>
-      <c r="J1">
+      <c r="K1">
         <v>2040</v>
       </c>
-      <c r="K1">
+      <c r="L1">
         <v>2045</v>
       </c>
-      <c r="L1">
+      <c r="M1">
         <v>2050</v>
       </c>
-      <c r="M1">
+      <c r="N1">
         <v>2055</v>
       </c>
-      <c r="N1">
+      <c r="O1">
         <v>2060</v>
       </c>
-      <c r="O1">
+      <c r="P1">
         <v>2065</v>
       </c>
-      <c r="P1">
+      <c r="Q1">
         <v>2070</v>
       </c>
-      <c r="Q1">
+      <c r="R1">
         <v>2075</v>
       </c>
-      <c r="R1">
+      <c r="S1">
         <v>2080</v>
       </c>
-      <c r="S1">
+      <c r="T1">
         <v>2085</v>
       </c>
-      <c r="T1">
+      <c r="U1">
         <v>2090</v>
       </c>
-      <c r="U1">
+      <c r="V1">
         <v>2095</v>
       </c>
-      <c r="V1">
+      <c r="W1">
         <v>2100</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>42369.982642000003</v>
+        <v>42369.982642</v>
       </c>
       <c r="D2">
-        <v>47284.947024000001</v>
+        <v>47284.947024</v>
       </c>
       <c r="E2">
-        <v>48382.783671999998</v>
+        <v>48382.783672</v>
       </c>
       <c r="F2">
-        <v>51570.022582999998</v>
+        <v>51570.022583</v>
       </c>
       <c r="G2">
-        <v>44786.450936000001</v>
+        <v>51570.022583</v>
       </c>
       <c r="H2">
-        <v>38002.836216999996</v>
+        <v>44786.450936</v>
       </c>
       <c r="I2">
-        <v>31219.317062999999</v>
+        <v>38002.836217</v>
       </c>
       <c r="J2">
-        <v>24436.372478000001</v>
+        <v>31219.317063</v>
       </c>
       <c r="K2">
+        <v>24436.372478</v>
+      </c>
+      <c r="L2">
         <v>17652.090676</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>10867.507806</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>4085.171996</v>
       </c>
-      <c r="N2">
-        <v>4.9890879999999997</v>
-      </c>
       <c r="O2">
-        <v>5.0154800000000002</v>
+        <v>4.989088</v>
       </c>
       <c r="P2">
-        <v>4.9956509999999996</v>
+        <v>5.01548</v>
       </c>
       <c r="Q2">
-        <v>4.9937909999999999</v>
+        <v>4.995651</v>
       </c>
       <c r="R2">
+        <v>4.993791</v>
+      </c>
+      <c r="S2">
         <v>4.991231</v>
       </c>
-      <c r="S2">
-        <v>5.0044409999999999</v>
-      </c>
       <c r="T2">
+        <v>5.004441</v>
+      </c>
+      <c r="U2">
         <v>4.998926</v>
       </c>
-      <c r="U2">
-        <v>-1.4596640000000001</v>
-      </c>
       <c r="V2">
-        <v>4.9973470000000004</v>
-      </c>
-      <c r="W2" t="s">
-        <v>17</v>
+        <v>-1.459664</v>
+      </c>
+      <c r="W2">
+        <v>4.997347</v>
+      </c>
+      <c r="X2" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C3">
-        <v>8406.4114399999999</v>
+        <v>8406.41144</v>
       </c>
       <c r="D3">
         <v>10678.65393</v>
@@ -620,285 +1199,297 @@
         <v>11973.88709</v>
       </c>
       <c r="F3">
-        <v>12508.934380000001</v>
+        <v>12508.93438</v>
       </c>
       <c r="G3">
-        <v>10841.133449999999</v>
+        <v>12508.93438</v>
       </c>
       <c r="H3">
-        <v>9706.8304900000003</v>
+        <v>10841.13345</v>
       </c>
       <c r="I3">
-        <v>6680.3603899999998</v>
+        <v>9706.83049</v>
       </c>
       <c r="J3">
-        <v>4188.8702800000001</v>
+        <v>6680.36039</v>
       </c>
       <c r="K3">
+        <v>4188.87028</v>
+      </c>
+      <c r="L3">
         <v>2681.471</v>
       </c>
-      <c r="L3">
-        <v>1754.0133499999999</v>
-      </c>
       <c r="M3">
+        <v>1754.01335</v>
+      </c>
+      <c r="N3">
         <v>1001.48068</v>
       </c>
-      <c r="N3">
-        <v>254.09111999999999</v>
-      </c>
       <c r="O3">
-        <v>-23.744810000000001</v>
+        <v>254.09112</v>
       </c>
       <c r="P3">
-        <v>-261.79984999999999</v>
+        <v>-23.74481</v>
       </c>
       <c r="Q3">
-        <v>-414.56065000000001</v>
+        <v>-261.79985</v>
       </c>
       <c r="R3">
-        <v>-507.28611999999998</v>
+        <v>-414.56065</v>
       </c>
       <c r="S3">
-        <v>-575.76374999999996</v>
+        <v>-507.28612</v>
       </c>
       <c r="T3">
+        <v>-575.76375</v>
+      </c>
+      <c r="U3">
         <v>-629.13986</v>
       </c>
-      <c r="U3">
-        <v>-627.19476999999995</v>
-      </c>
       <c r="V3">
-        <v>-607.35677999999996</v>
-      </c>
-      <c r="W3" t="s">
-        <v>17</v>
+        <v>-627.19477</v>
+      </c>
+      <c r="W3">
+        <v>-607.35678</v>
+      </c>
+      <c r="X3" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C4">
         <v>30561.83</v>
       </c>
       <c r="D4">
-        <v>34332.793100000003</v>
+        <v>34332.7931</v>
       </c>
       <c r="E4">
-        <v>34193.253700000001</v>
+        <v>34193.2537</v>
       </c>
       <c r="F4">
-        <v>37615.253700000001</v>
+        <v>37615.2537</v>
       </c>
       <c r="G4">
-        <v>33404.437599999997</v>
+        <v>37615.2537</v>
       </c>
       <c r="H4">
+        <v>33404.4376</v>
+      </c>
+      <c r="I4">
         <v>26934.9143</v>
       </c>
-      <c r="I4">
-        <v>20127.896400000001</v>
-      </c>
       <c r="J4">
-        <v>13253.325500000001</v>
+        <v>20127.8964</v>
       </c>
       <c r="K4">
-        <v>6469.6590999999999</v>
+        <v>13253.3255</v>
       </c>
       <c r="L4">
+        <v>6469.6591</v>
+      </c>
+      <c r="M4">
         <v>-194.3725</v>
       </c>
-      <c r="M4">
-        <v>-6559.0658999999996</v>
-      </c>
       <c r="N4">
-        <v>-10252.487999999999</v>
+        <v>-6559.0659</v>
       </c>
       <c r="O4">
+        <v>-10252.488</v>
+      </c>
+      <c r="P4">
         <v>-10559.9787</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>-10728.6446</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>-10877.7968</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>-10997.7971</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>-11115.1363</v>
       </c>
-      <c r="T4">
-        <v>-11227.301799999999</v>
-      </c>
       <c r="U4">
+        <v>-11227.3018</v>
+      </c>
+      <c r="V4">
         <v>-11360.7552</v>
       </c>
-      <c r="V4">
-        <v>-11489.622799999999</v>
-      </c>
-      <c r="W4" t="s">
-        <v>18</v>
+      <c r="W4">
+        <v>-11489.6228</v>
+      </c>
+      <c r="X4" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24">
       <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5">
+        <v>29385.90388</v>
+      </c>
+      <c r="D5">
+        <v>32646.60704</v>
+      </c>
+      <c r="E5">
+        <v>37123.69377</v>
+      </c>
+      <c r="F5">
+        <v>40119.18767</v>
+      </c>
+      <c r="G5">
+        <v>40119.18767</v>
+      </c>
+      <c r="H5">
+        <v>36508.5539</v>
+      </c>
+      <c r="I5">
+        <v>30735.08394</v>
+      </c>
+      <c r="J5">
+        <v>22622.77614</v>
+      </c>
+      <c r="K5">
+        <v>14184.36004</v>
+      </c>
+      <c r="L5">
+        <v>5899.80606</v>
+      </c>
+      <c r="M5">
+        <v>-42.27179</v>
+      </c>
+      <c r="N5">
+        <v>-4874.37045</v>
+      </c>
+      <c r="O5">
+        <v>-8003.28093</v>
+      </c>
+      <c r="P5">
+        <v>-8256.27167</v>
+      </c>
+      <c r="Q5">
+        <v>-8772.3775</v>
+      </c>
+      <c r="R5">
+        <v>-9191.48351</v>
+      </c>
+      <c r="S5">
+        <v>-9514.56406</v>
+      </c>
+      <c r="T5">
+        <v>-9777.60146</v>
+      </c>
+      <c r="U5">
+        <v>-10013.38839</v>
+      </c>
+      <c r="V5">
+        <v>-10268.94062</v>
+      </c>
+      <c r="W5">
+        <v>-10525.09104</v>
+      </c>
+      <c r="X5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:24">
+      <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="C5">
-        <v>29385.903880000002</v>
-      </c>
-      <c r="D5">
-        <v>32646.607039999999</v>
-      </c>
-      <c r="E5">
-        <v>37123.693769999998</v>
-      </c>
-      <c r="F5">
-        <v>40119.187669999999</v>
-      </c>
-      <c r="G5">
-        <v>36508.553899999999</v>
-      </c>
-      <c r="H5">
-        <v>30735.08394</v>
-      </c>
-      <c r="I5">
-        <v>22622.776140000002</v>
-      </c>
-      <c r="J5">
-        <v>14184.36004</v>
-      </c>
-      <c r="K5">
-        <v>5899.8060599999999</v>
-      </c>
-      <c r="L5">
-        <v>-42.271790000000003</v>
-      </c>
-      <c r="M5">
-        <v>-4874.3704500000003</v>
-      </c>
-      <c r="N5">
-        <v>-8003.2809299999999</v>
-      </c>
-      <c r="O5">
-        <v>-8256.2716700000001</v>
-      </c>
-      <c r="P5">
-        <v>-8772.3775000000005</v>
-      </c>
-      <c r="Q5">
-        <v>-9191.48351</v>
-      </c>
-      <c r="R5">
-        <v>-9514.5640600000006</v>
-      </c>
-      <c r="S5">
-        <v>-9777.6014599999999</v>
-      </c>
-      <c r="T5">
-        <v>-10013.38839</v>
-      </c>
-      <c r="U5">
-        <v>-10268.940619999999</v>
-      </c>
-      <c r="V5">
-        <v>-10525.091039999999</v>
-      </c>
-      <c r="W5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C6">
-        <v>6531.7096700000002</v>
+        <v>6531.70967</v>
       </c>
       <c r="D6">
-        <v>8494.4172799999997</v>
+        <v>8494.41728</v>
       </c>
       <c r="E6">
         <v>10052.30409</v>
       </c>
       <c r="F6">
-        <v>10753.726650000001</v>
+        <v>10753.72665</v>
       </c>
       <c r="G6">
-        <v>9529.7436099999995</v>
+        <v>10753.72665</v>
       </c>
       <c r="H6">
-        <v>8468.5824400000001</v>
+        <v>9529.74361</v>
       </c>
       <c r="I6">
-        <v>5475.5743700000003</v>
+        <v>8468.58244</v>
       </c>
       <c r="J6">
-        <v>3017.0236599999998</v>
+        <v>5475.57437</v>
       </c>
       <c r="K6">
-        <v>1551.2339999999999</v>
+        <v>3017.02366</v>
       </c>
       <c r="L6">
-        <v>675.35766000000001</v>
+        <v>1551.234</v>
       </c>
       <c r="M6">
-        <v>-27.358740000000001</v>
+        <v>675.35766</v>
       </c>
       <c r="N6">
-        <v>-694.99186999999995</v>
+        <v>-27.35874</v>
       </c>
       <c r="O6">
-        <v>-968.49940000000004</v>
+        <v>-694.99187</v>
       </c>
       <c r="P6">
+        <v>-968.4994</v>
+      </c>
+      <c r="Q6">
         <v>-1176.86094</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>-1302.83663</v>
       </c>
-      <c r="R6">
-        <v>-1367.8017500000001</v>
-      </c>
       <c r="S6">
-        <v>-1408.2004199999999</v>
+        <v>-1367.80175</v>
       </c>
       <c r="T6">
-        <v>-1433.4540400000001</v>
+        <v>-1408.20042</v>
       </c>
       <c r="U6">
-        <v>-1409.4985799999999</v>
+        <v>-1433.45404</v>
       </c>
       <c r="V6">
+        <v>-1409.49858</v>
+      </c>
+      <c r="W6">
         <v>-1363.93613</v>
       </c>
-      <c r="W6" t="s">
-        <v>18</v>
+      <c r="X6" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C7">
-        <v>6471.3837999999996</v>
+        <v>6471.3838</v>
       </c>
       <c r="D7">
-        <v>8745.7739000000001</v>
+        <v>8745.7739</v>
       </c>
       <c r="E7">
         <v>10353.9894</v>
@@ -907,347 +1498,362 @@
         <v>10995.4087</v>
       </c>
       <c r="G7">
-        <v>9765.2507999999998</v>
+        <v>10995.4087</v>
       </c>
       <c r="H7">
-        <v>8772.5069999999996</v>
+        <v>9765.2508</v>
       </c>
       <c r="I7">
+        <v>8772.507</v>
+      </c>
+      <c r="J7">
         <v>5787.0944</v>
       </c>
-      <c r="J7">
-        <v>3310.5111999999999</v>
-      </c>
       <c r="K7">
+        <v>3310.5112</v>
+      </c>
+      <c r="L7">
         <v>1835.15</v>
       </c>
-      <c r="L7">
-        <v>979.20510000000002</v>
-      </c>
       <c r="M7">
+        <v>979.2051</v>
+      </c>
+      <c r="N7">
         <v>266.2004</v>
       </c>
-      <c r="N7">
-        <v>-380.28039999999999</v>
-      </c>
       <c r="O7">
-        <v>-662.80029999999999</v>
+        <v>-380.2804</v>
       </c>
       <c r="P7">
-        <v>-905.17660000000001</v>
+        <v>-662.8003</v>
       </c>
       <c r="Q7">
+        <v>-905.1766</v>
+      </c>
+      <c r="R7">
         <v>-1057.7699</v>
       </c>
-      <c r="R7">
-        <v>-1143.0328999999999</v>
-      </c>
       <c r="S7">
-        <v>-1197.3825999999999</v>
+        <v>-1143.0329</v>
       </c>
       <c r="T7">
-        <v>-1232.8710000000001</v>
+        <v>-1197.3826</v>
       </c>
       <c r="U7">
+        <v>-1232.871</v>
+      </c>
+      <c r="V7">
         <v>-1217.4412</v>
       </c>
-      <c r="V7">
-        <v>-1180.0360000000001</v>
-      </c>
-      <c r="W7" t="s">
-        <v>18</v>
+      <c r="W7">
+        <v>-1180.036</v>
+      </c>
+      <c r="X7" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C8">
-        <v>2541.1350000000002</v>
+        <v>2541.135</v>
       </c>
       <c r="D8">
-        <v>4246.8239999999996</v>
+        <v>4246.824</v>
       </c>
       <c r="E8">
         <v>5443.79</v>
       </c>
       <c r="F8">
-        <v>6621.8220000000001</v>
+        <v>6621.822</v>
       </c>
       <c r="G8">
-        <v>7533.8950000000004</v>
+        <v>6621.822</v>
       </c>
       <c r="H8">
-        <v>9399.0789999999997</v>
+        <v>7533.895</v>
       </c>
       <c r="I8">
+        <v>9399.079</v>
+      </c>
+      <c r="J8">
         <v>11873.547</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>14388.355</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>16616.62</v>
       </c>
-      <c r="L8">
-        <v>18282.441999999999</v>
-      </c>
       <c r="M8">
-        <v>19181.085999999999</v>
+        <v>18282.442</v>
       </c>
       <c r="N8">
-        <v>19906.004000000001</v>
+        <v>19181.086</v>
       </c>
       <c r="O8">
-        <v>19653.809000000001</v>
+        <v>19906.004</v>
       </c>
       <c r="P8">
-        <v>19424.683000000001</v>
+        <v>19653.809</v>
       </c>
       <c r="Q8">
+        <v>19424.683</v>
+      </c>
+      <c r="R8">
         <v>18946.197</v>
       </c>
-      <c r="R8">
-        <v>18426.939999999999</v>
-      </c>
       <c r="S8">
-        <v>17835.745999999999</v>
+        <v>18426.94</v>
       </c>
       <c r="T8">
-        <v>17218.022000000001</v>
+        <v>17835.746</v>
       </c>
       <c r="U8">
-        <v>16589.363000000001</v>
+        <v>17218.022</v>
       </c>
       <c r="V8">
+        <v>16589.363</v>
+      </c>
+      <c r="W8">
         <v>16041.724</v>
       </c>
-      <c r="W8" t="s">
-        <v>19</v>
+      <c r="X8" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C9" s="1">
         <v>2001.721</v>
       </c>
       <c r="D9" s="1">
-        <v>3296.4760000000001</v>
+        <v>3296.476</v>
       </c>
       <c r="E9" s="1">
-        <v>3996.4389999999999</v>
+        <v>3996.439</v>
       </c>
       <c r="F9" s="1">
-        <v>4332.4009999999998</v>
+        <v>4332.401</v>
       </c>
       <c r="G9" s="1">
-        <v>3873.6950000000002</v>
+        <v>4332.401</v>
       </c>
       <c r="H9" s="1">
+        <v>3873.695</v>
+      </c>
+      <c r="I9" s="1">
         <v>3675.96</v>
       </c>
-      <c r="I9" s="1">
-        <v>1766.5360000000001</v>
-      </c>
       <c r="J9" s="1">
-        <v>343.59879999999998</v>
+        <v>1766.536</v>
       </c>
       <c r="K9" s="1">
-        <v>25.069839999999999</v>
+        <v>343.5988</v>
       </c>
       <c r="L9" s="1">
-        <v>3.1127750000000001</v>
+        <v>25.06984</v>
       </c>
       <c r="M9" s="1">
-        <v>0.30459570000000002</v>
+        <v>3.112775</v>
       </c>
       <c r="N9" s="1">
-        <v>1.9324520000000001E-2</v>
+        <v>0.3045957</v>
       </c>
       <c r="O9" s="1">
-        <v>1.9198349999999999E-2</v>
+        <v>0.01932452</v>
       </c>
       <c r="P9" s="1">
-        <v>1.2645190000000001E-2</v>
+        <v>0.01919835</v>
       </c>
       <c r="Q9" s="1">
-        <v>5.7631410000000003E-3</v>
+        <v>0.01264519</v>
       </c>
       <c r="R9" s="1">
-        <v>2.7393259999999998E-3</v>
+        <v>0.005763141</v>
       </c>
       <c r="S9" s="1">
-        <v>1.315711E-3</v>
+        <v>0.002739326</v>
       </c>
       <c r="T9" s="1">
-        <v>4.2004199999999997E-4</v>
+        <v>0.001315711</v>
       </c>
       <c r="U9" s="1">
-        <v>6.2735970000000002E-5</v>
+        <v>0.000420042</v>
       </c>
       <c r="V9" s="1">
-        <v>8.6114259999999997E-6</v>
-      </c>
-      <c r="W9" t="s">
-        <v>19</v>
+        <v>6.273597e-5</v>
+      </c>
+      <c r="W9" s="1">
+        <v>8.611426e-6</v>
+      </c>
+      <c r="X9" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C10">
-        <v>0.95913800000000005</v>
+        <v>0.959138</v>
       </c>
       <c r="D10">
-        <v>1.0983799999999999</v>
+        <v>1.09838</v>
       </c>
       <c r="E10">
         <v>1.24343</v>
       </c>
       <c r="F10">
-        <v>1.3521300000000001</v>
+        <v>1.35213</v>
       </c>
       <c r="G10">
+        <v>1.35213</v>
+      </c>
+      <c r="H10">
         <v>1.45913</v>
       </c>
-      <c r="H10">
-        <v>1.5742100000000001</v>
-      </c>
       <c r="I10">
-        <v>1.6798900000000001</v>
+        <v>1.57421</v>
       </c>
       <c r="J10">
-        <v>1.7730600000000001</v>
+        <v>1.67989</v>
       </c>
       <c r="K10">
-        <v>1.8477600000000001</v>
+        <v>1.77306</v>
       </c>
       <c r="L10">
+        <v>1.84776</v>
+      </c>
+      <c r="M10">
         <v>1.92377</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>1.98089</v>
       </c>
-      <c r="N10">
-        <v>1.9963900000000001</v>
-      </c>
       <c r="O10">
+        <v>1.99639</v>
+      </c>
+      <c r="P10">
         <v>1.98444</v>
       </c>
-      <c r="P10">
-        <v>1.9577500000000001</v>
-      </c>
       <c r="Q10">
-        <v>1.9111400000000001</v>
+        <v>1.95775</v>
       </c>
       <c r="R10">
+        <v>1.91114</v>
+      </c>
+      <c r="S10">
         <v>1.84643</v>
       </c>
-      <c r="S10">
-        <v>1.7707900000000001</v>
-      </c>
       <c r="T10">
-        <v>1.6955100000000001</v>
+        <v>1.77079</v>
       </c>
       <c r="U10">
-        <v>1.6284700000000001</v>
+        <v>1.69551</v>
       </c>
       <c r="V10">
-        <v>1.5708899999999999</v>
-      </c>
-      <c r="W10" t="s">
-        <v>20</v>
+        <v>1.62847</v>
+      </c>
+      <c r="W10">
+        <v>1.57089</v>
+      </c>
+      <c r="X10" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C11">
-        <v>2.1581000000000001</v>
+        <v>2.1581</v>
       </c>
       <c r="D11">
-        <v>2.3890899999999999</v>
+        <v>2.38909</v>
       </c>
       <c r="E11">
-        <v>2.6120299999999999</v>
+        <v>2.61203</v>
       </c>
       <c r="F11">
         <v>2.79257</v>
       </c>
       <c r="G11">
+        <v>2.79257</v>
+      </c>
+      <c r="H11">
         <v>2.96875</v>
       </c>
-      <c r="H11">
-        <v>3.1108099999999999</v>
-      </c>
       <c r="I11">
-        <v>3.1941899999999999</v>
+        <v>3.11081</v>
       </c>
       <c r="J11">
-        <v>3.2153999999999998</v>
+        <v>3.19419</v>
       </c>
       <c r="K11">
+        <v>3.2154</v>
+      </c>
+      <c r="L11">
         <v>3.16134</v>
       </c>
-      <c r="L11">
-        <v>3.0654699999999999</v>
-      </c>
       <c r="M11">
+        <v>3.06547</v>
+      </c>
+      <c r="N11">
         <v>2.94055</v>
       </c>
-      <c r="N11">
-        <v>2.7813599999999998</v>
-      </c>
       <c r="O11">
-        <v>2.6202700000000001</v>
+        <v>2.78136</v>
       </c>
       <c r="P11">
-        <v>2.4923099999999998</v>
+        <v>2.62027</v>
       </c>
       <c r="Q11">
-        <v>2.3863400000000001</v>
+        <v>2.49231</v>
       </c>
       <c r="R11">
-        <v>2.2965200000000001</v>
+        <v>2.38634</v>
       </c>
       <c r="S11">
-        <v>2.2180200000000001</v>
+        <v>2.29652</v>
       </c>
       <c r="T11">
+        <v>2.21802</v>
+      </c>
+      <c r="U11">
         <v>2.14859</v>
       </c>
-      <c r="U11">
+      <c r="V11">
         <v>2.08623</v>
       </c>
-      <c r="V11">
+      <c r="W11">
         <v>2.0301</v>
       </c>
-      <c r="W11" t="s">
-        <v>21</v>
+      <c r="X11" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1259,143 +1865,149 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>4.5325749999999996</v>
+        <v>4.532575</v>
       </c>
       <c r="G12">
-        <v>55.276454800000003</v>
+        <v>4.532575</v>
       </c>
       <c r="H12">
+        <v>55.2764548</v>
+      </c>
+      <c r="I12">
         <v>101.7579298</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>142.7051472</v>
       </c>
-      <c r="J12">
-        <v>206.11676170000001</v>
-      </c>
       <c r="K12">
-        <v>322.56643680000002</v>
+        <v>206.1167617</v>
       </c>
       <c r="L12">
+        <v>322.5664368</v>
+      </c>
+      <c r="M12">
         <v>439.9639962</v>
       </c>
-      <c r="M12">
-        <v>652.01035260000003</v>
-      </c>
       <c r="N12">
+        <v>652.0103526</v>
+      </c>
+      <c r="O12">
         <v>1049.7703755</v>
       </c>
-      <c r="O12">
-        <v>1045.2528973000001</v>
-      </c>
       <c r="P12">
-        <v>1114.3189887999999</v>
+        <v>1045.2528973</v>
       </c>
       <c r="Q12">
-        <v>1177.9428370000001</v>
+        <v>1114.3189888</v>
       </c>
       <c r="R12">
-        <v>1246.5188029999999</v>
+        <v>1177.942837</v>
       </c>
       <c r="S12">
-        <v>1303.0681970999999</v>
+        <v>1246.518803</v>
       </c>
       <c r="T12">
+        <v>1303.0681971</v>
+      </c>
+      <c r="U12">
         <v>1358.9702556</v>
       </c>
-      <c r="U12">
-        <v>1421.6878337999999</v>
-      </c>
       <c r="V12">
-        <v>1484.6134841999999</v>
-      </c>
-      <c r="W12" t="s">
-        <v>22</v>
+        <v>1421.6878338</v>
+      </c>
+      <c r="W12">
+        <v>1484.6134842</v>
+      </c>
+      <c r="X12" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C13">
-        <v>42369.982642000003</v>
+        <v>42369.982642</v>
       </c>
       <c r="D13">
-        <v>47284.947024000001</v>
+        <v>47284.947024</v>
       </c>
       <c r="E13">
-        <v>48382.783671999998</v>
+        <v>48382.783672</v>
       </c>
       <c r="F13">
-        <v>51570.022582999998</v>
+        <v>51570.022583</v>
       </c>
       <c r="G13">
-        <v>47664.257602999998</v>
+        <v>51570.022583</v>
       </c>
       <c r="H13">
-        <v>43758.636031000002</v>
+        <v>47664.257603</v>
       </c>
       <c r="I13">
-        <v>39852.820720999996</v>
+        <v>43758.636031</v>
       </c>
       <c r="J13">
-        <v>35947.271410000001</v>
+        <v>39852.820721</v>
       </c>
       <c r="K13">
-        <v>32061.304843000002</v>
+        <v>35947.27141</v>
       </c>
       <c r="L13">
-        <v>28135.971348999999</v>
+        <v>32061.304843</v>
       </c>
       <c r="M13">
-        <v>24225.590099000001</v>
+        <v>28135.971349</v>
       </c>
       <c r="N13">
-        <v>20324.547178000001</v>
+        <v>24225.590099</v>
       </c>
       <c r="O13">
+        <v>20324.547178</v>
+      </c>
+      <c r="P13">
         <v>16419.132126</v>
       </c>
-      <c r="P13">
-        <v>12513.180044000001</v>
-      </c>
       <c r="Q13">
-        <v>8607.4908149999992</v>
+        <v>12513.180044</v>
       </c>
       <c r="R13">
+        <v>8607.490815</v>
+      </c>
+      <c r="S13">
         <v>4702.02286</v>
       </c>
-      <c r="S13">
-        <v>796.13876200000004</v>
-      </c>
       <c r="T13">
-        <v>4.9838019999999998</v>
+        <v>796.138762</v>
       </c>
       <c r="U13">
-        <v>4.9920520000000002</v>
+        <v>4.983802</v>
       </c>
       <c r="V13">
-        <v>4.9964440000000003</v>
-      </c>
-      <c r="W13" t="s">
-        <v>17</v>
+        <v>4.992052</v>
+      </c>
+      <c r="W13">
+        <v>4.996444</v>
+      </c>
+      <c r="X13" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C14">
-        <v>8406.4114000000009</v>
+        <v>8406.4114</v>
       </c>
       <c r="D14">
-        <v>10678.653899999999</v>
+        <v>10678.6539</v>
       </c>
       <c r="E14">
         <v>11973.8871</v>
@@ -1404,282 +2016,294 @@
         <v>12508.9344</v>
       </c>
       <c r="G14">
-        <v>11628.028200000001</v>
+        <v>12508.9344</v>
       </c>
       <c r="H14">
-        <v>11068.630499999999</v>
+        <v>11628.0282</v>
       </c>
       <c r="I14">
-        <v>9518.7872000000007</v>
+        <v>11068.6305</v>
       </c>
       <c r="J14">
-        <v>7799.3747000000003</v>
+        <v>9518.7872</v>
       </c>
       <c r="K14">
+        <v>7799.3747</v>
+      </c>
+      <c r="L14">
         <v>6200.3732</v>
       </c>
-      <c r="L14">
-        <v>4822.4504999999999</v>
-      </c>
       <c r="M14">
-        <v>3589.0666999999999</v>
+        <v>4822.4505</v>
       </c>
       <c r="N14">
-        <v>2684.6406000000002</v>
+        <v>3589.0667</v>
       </c>
       <c r="O14">
-        <v>1988.7398000000001</v>
+        <v>2684.6406</v>
       </c>
       <c r="P14">
-        <v>1426.3503000000001</v>
+        <v>1988.7398</v>
       </c>
       <c r="Q14">
-        <v>981.53740000000005</v>
+        <v>1426.3503</v>
       </c>
       <c r="R14">
-        <v>418.92680000000001</v>
+        <v>981.5374</v>
       </c>
       <c r="S14">
+        <v>418.9268</v>
+      </c>
+      <c r="T14">
         <v>-155.6277</v>
       </c>
-      <c r="T14">
-        <v>-330.39589999999998</v>
-      </c>
       <c r="U14">
-        <v>-461.94209999999998</v>
+        <v>-330.3959</v>
       </c>
       <c r="V14">
-        <v>-537.20799999999997</v>
-      </c>
-      <c r="W14" t="s">
-        <v>17</v>
+        <v>-461.9421</v>
+      </c>
+      <c r="W14">
+        <v>-537.208</v>
+      </c>
+      <c r="X14" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C15">
         <v>30561.83</v>
       </c>
       <c r="D15">
-        <v>34332.793100000003</v>
+        <v>34332.7931</v>
       </c>
       <c r="E15">
-        <v>34193.253700000001</v>
+        <v>34193.2537</v>
       </c>
       <c r="F15">
-        <v>37615.253700000001</v>
+        <v>37615.2537</v>
       </c>
       <c r="G15">
-        <v>35740.673900000002</v>
+        <v>37615.2537</v>
       </c>
       <c r="H15">
-        <v>32199.433700000001</v>
+        <v>35740.6739</v>
       </c>
       <c r="I15">
-        <v>28294.307199999999</v>
+        <v>32199.4337</v>
       </c>
       <c r="J15">
-        <v>24200.783299999999</v>
+        <v>28294.3072</v>
       </c>
       <c r="K15">
-        <v>20106.952399999998</v>
+        <v>24200.7833</v>
       </c>
       <c r="L15">
+        <v>20106.9524</v>
+      </c>
+      <c r="M15">
         <v>16087.1579</v>
       </c>
-      <c r="M15">
-        <v>12189.456399999999</v>
-      </c>
       <c r="N15">
-        <v>8290.9169999999995</v>
+        <v>12189.4564</v>
       </c>
       <c r="O15">
+        <v>8290.917</v>
+      </c>
+      <c r="P15">
         <v>4370.9946</v>
       </c>
-      <c r="P15">
-        <v>477.49939999999998</v>
-      </c>
       <c r="Q15">
-        <v>-3270.5821999999998</v>
+        <v>477.4994</v>
       </c>
       <c r="R15">
-        <v>-6734.1027999999997</v>
+        <v>-3270.5822</v>
       </c>
       <c r="S15">
-        <v>-10311.856599999999</v>
+        <v>-6734.1028</v>
       </c>
       <c r="T15">
-        <v>-11316.680700000001</v>
+        <v>-10311.8566</v>
       </c>
       <c r="U15">
+        <v>-11316.6807</v>
+      </c>
+      <c r="V15">
         <v>-11473.1873</v>
       </c>
-      <c r="V15">
+      <c r="W15">
         <v>-11581.7256</v>
       </c>
-      <c r="W15" t="s">
-        <v>18</v>
+      <c r="X15" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24">
       <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
         <v>9</v>
       </c>
-      <c r="B16" t="s">
-        <v>3</v>
-      </c>
       <c r="C16">
-        <v>29385.903999999999</v>
+        <v>29385.904</v>
       </c>
       <c r="D16">
         <v>32646.607</v>
       </c>
       <c r="E16">
-        <v>37123.694000000003</v>
+        <v>37123.694</v>
       </c>
       <c r="F16">
-        <v>40119.188000000002</v>
+        <v>40119.188</v>
       </c>
       <c r="G16">
-        <v>38678.635999999999</v>
+        <v>40119.188</v>
       </c>
       <c r="H16">
-        <v>35600.656000000003</v>
+        <v>38678.636</v>
       </c>
       <c r="I16">
-        <v>31009.133999999998</v>
+        <v>35600.656</v>
       </c>
       <c r="J16">
-        <v>25923.825000000001</v>
+        <v>31009.134</v>
       </c>
       <c r="K16">
-        <v>21500.951000000001</v>
+        <v>25923.825</v>
       </c>
       <c r="L16">
+        <v>21500.951</v>
+      </c>
+      <c r="M16">
         <v>17487.607</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <v>13246.704</v>
       </c>
-      <c r="N16">
-        <v>8709.8790000000008</v>
-      </c>
       <c r="O16">
+        <v>8709.879</v>
+      </c>
+      <c r="P16">
         <v>4094.145</v>
       </c>
-      <c r="P16">
+      <c r="Q16">
         <v>-107.718</v>
       </c>
-      <c r="Q16">
-        <v>-2291.1860000000001</v>
-      </c>
       <c r="R16">
-        <v>-5477.2860000000001</v>
+        <v>-2291.186</v>
       </c>
       <c r="S16">
-        <v>-8672.4120000000003</v>
+        <v>-5477.286</v>
       </c>
       <c r="T16">
-        <v>-9166.7929999999997</v>
+        <v>-8672.412</v>
       </c>
       <c r="U16">
-        <v>-9620.7270000000008</v>
+        <v>-9166.793</v>
       </c>
       <c r="V16">
-        <v>-10049.217000000001</v>
-      </c>
-      <c r="W16" t="s">
-        <v>18</v>
+        <v>-9620.727</v>
+      </c>
+      <c r="W16">
+        <v>-10049.217</v>
+      </c>
+      <c r="X16" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C17">
-        <v>6531.7096700000002</v>
+        <v>6531.70967</v>
       </c>
       <c r="D17">
-        <v>8494.4172799999997</v>
+        <v>8494.41728</v>
       </c>
       <c r="E17">
         <v>10052.30409</v>
       </c>
       <c r="F17">
-        <v>10753.726650000001</v>
+        <v>10753.72665</v>
       </c>
       <c r="G17">
+        <v>10753.72665</v>
+      </c>
+      <c r="H17">
         <v>10175.4992</v>
       </c>
-      <c r="H17">
-        <v>9733.7319299999999</v>
-      </c>
       <c r="I17">
-        <v>8202.5040200000003</v>
+        <v>9733.73193</v>
       </c>
       <c r="J17">
-        <v>6541.0340800000004</v>
+        <v>8202.50402</v>
       </c>
       <c r="K17">
-        <v>4987.4449500000001</v>
+        <v>6541.03408</v>
       </c>
       <c r="L17">
-        <v>3665.0487800000001</v>
+        <v>4987.44495</v>
       </c>
       <c r="M17">
-        <v>2463.9731099999999</v>
+        <v>3665.04878</v>
       </c>
       <c r="N17">
+        <v>2463.97311</v>
+      </c>
+      <c r="O17">
         <v>1599.13696</v>
       </c>
-      <c r="O17">
-        <v>942.72553000000005</v>
-      </c>
       <c r="P17">
+        <v>942.72553</v>
+      </c>
+      <c r="Q17">
         <v>418.75151</v>
       </c>
-      <c r="Q17">
+      <c r="R17">
         <v>12.43704</v>
       </c>
-      <c r="R17">
-        <v>-483.17919999999998</v>
-      </c>
       <c r="S17">
-        <v>-991.15144999999995</v>
+        <v>-483.1792</v>
       </c>
       <c r="T17">
+        <v>-991.15145</v>
+      </c>
+      <c r="U17">
         <v>-1152.22525</v>
       </c>
-      <c r="U17">
-        <v>-1238.1376700000001</v>
-      </c>
       <c r="V17">
+        <v>-1238.13767</v>
+      </c>
+      <c r="W17">
         <v>-1284.72966</v>
       </c>
-      <c r="W17" t="s">
-        <v>18</v>
+      <c r="X17" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C18">
-        <v>6471.3837999999996</v>
+        <v>6471.3838</v>
       </c>
       <c r="D18">
-        <v>8745.7739000000001</v>
+        <v>8745.7739</v>
       </c>
       <c r="E18">
         <v>10353.9894</v>
@@ -1688,347 +2312,362 @@
         <v>10995.4087</v>
       </c>
       <c r="G18">
-        <v>10410.421200000001</v>
+        <v>10995.4087</v>
       </c>
       <c r="H18">
+        <v>10410.4212</v>
+      </c>
+      <c r="I18">
         <v>10013.2894</v>
       </c>
-      <c r="I18">
-        <v>8488.9945000000007</v>
-      </c>
       <c r="J18">
-        <v>6814.5191000000004</v>
+        <v>8488.9945</v>
       </c>
       <c r="K18">
-        <v>5257.3379999999997</v>
+        <v>6814.5191</v>
       </c>
       <c r="L18">
-        <v>3930.1194999999998</v>
+        <v>5257.338</v>
       </c>
       <c r="M18">
-        <v>2697.8395999999998</v>
+        <v>3930.1195</v>
       </c>
       <c r="N18">
+        <v>2697.8396</v>
+      </c>
+      <c r="O18">
         <v>1813.3477</v>
       </c>
-      <c r="O18">
+      <c r="P18">
         <v>1142.7655</v>
       </c>
-      <c r="P18">
-        <v>601.05110000000002</v>
-      </c>
       <c r="Q18">
-        <v>205.31890000000001</v>
+        <v>601.0511</v>
       </c>
       <c r="R18">
-        <v>-269.60879999999997</v>
+        <v>205.3189</v>
       </c>
       <c r="S18">
-        <v>-715.65039999999999</v>
+        <v>-269.6088</v>
       </c>
       <c r="T18">
-        <v>-858.49339999999995</v>
+        <v>-715.6504</v>
       </c>
       <c r="U18">
-        <v>-969.72900000000004</v>
+        <v>-858.4934</v>
       </c>
       <c r="V18">
+        <v>-969.729</v>
+      </c>
+      <c r="W18">
         <v>-1043.412</v>
       </c>
-      <c r="W18" t="s">
-        <v>18</v>
+      <c r="X18" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C19">
-        <v>2541.1350000000002</v>
+        <v>2541.135</v>
       </c>
       <c r="D19">
-        <v>4246.8239999999996</v>
+        <v>4246.824</v>
       </c>
       <c r="E19">
         <v>5443.79</v>
       </c>
       <c r="F19">
-        <v>6621.8220000000001</v>
+        <v>6621.822</v>
       </c>
       <c r="G19">
-        <v>7824.8959999999997</v>
+        <v>6621.822</v>
       </c>
       <c r="H19">
-        <v>8820.3739999999998</v>
+        <v>7824.896</v>
       </c>
       <c r="I19">
-        <v>10565.147000000001</v>
+        <v>8820.374</v>
       </c>
       <c r="J19">
+        <v>10565.147</v>
+      </c>
+      <c r="K19">
         <v>12262.401</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>13506.75</v>
       </c>
-      <c r="L19">
+      <c r="M19">
         <v>14839.564</v>
       </c>
-      <c r="M19">
+      <c r="N19">
         <v>15790.804</v>
       </c>
-      <c r="N19">
-        <v>16660.830000000002</v>
-      </c>
       <c r="O19">
+        <v>16660.83</v>
+      </c>
+      <c r="P19">
         <v>17145.234</v>
       </c>
-      <c r="P19">
-        <v>17322.271000000001</v>
-      </c>
       <c r="Q19">
-        <v>17106.403999999999</v>
+        <v>17322.271</v>
       </c>
       <c r="R19">
-        <v>17265.800999999999</v>
+        <v>17106.404</v>
       </c>
       <c r="S19">
-        <v>17285.187999999998</v>
+        <v>17265.801</v>
       </c>
       <c r="T19">
-        <v>16824.903999999999</v>
+        <v>17285.188</v>
       </c>
       <c r="U19">
-        <v>16348.326999999999</v>
+        <v>16824.904</v>
       </c>
       <c r="V19">
+        <v>16348.327</v>
+      </c>
+      <c r="W19">
         <v>15905.472</v>
       </c>
-      <c r="W19" t="s">
-        <v>19</v>
+      <c r="X19" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24">
       <c r="A20" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C20" s="1">
         <v>2001.721</v>
       </c>
       <c r="D20" s="1">
-        <v>3296.4760000000001</v>
+        <v>3296.476</v>
       </c>
       <c r="E20" s="1">
-        <v>3996.4389999999999</v>
+        <v>3996.439</v>
       </c>
       <c r="F20" s="1">
-        <v>4332.4009999999998</v>
+        <v>4332.401</v>
       </c>
       <c r="G20" s="1">
-        <v>4195.1239999999998</v>
+        <v>4332.401</v>
       </c>
       <c r="H20" s="1">
-        <v>4164.6660000000002</v>
+        <v>4195.124</v>
       </c>
       <c r="I20" s="1">
-        <v>3462.1770000000001</v>
+        <v>4164.666</v>
       </c>
       <c r="J20" s="1">
-        <v>2414.4589999999998</v>
+        <v>3462.177</v>
       </c>
       <c r="K20" s="1">
-        <v>1435.0550000000001</v>
+        <v>2414.459</v>
       </c>
       <c r="L20" s="1">
-        <v>693.07569999999998</v>
+        <v>1435.055</v>
       </c>
       <c r="M20" s="1">
-        <v>206.09790000000001</v>
+        <v>693.0757</v>
       </c>
       <c r="N20" s="1">
-        <v>42.895479999999999</v>
+        <v>206.0979</v>
       </c>
       <c r="O20" s="1">
+        <v>42.89548</v>
+      </c>
+      <c r="P20" s="1">
         <v>8.303172</v>
       </c>
-      <c r="P20" s="1">
-        <v>2.0896509999999999</v>
-      </c>
       <c r="Q20" s="1">
-        <v>0.63341020000000003</v>
+        <v>2.089651</v>
       </c>
       <c r="R20" s="1">
-        <v>4.5921669999999998E-2</v>
+        <v>0.6334102</v>
       </c>
       <c r="S20" s="1">
-        <v>1.864833E-3</v>
+        <v>0.04592167</v>
       </c>
       <c r="T20" s="1">
-        <v>1.6080630000000001E-3</v>
+        <v>0.001864833</v>
       </c>
       <c r="U20" s="1">
-        <v>7.8310339999999997E-4</v>
+        <v>0.001608063</v>
       </c>
       <c r="V20" s="1">
-        <v>2.7341650000000002E-4</v>
-      </c>
-      <c r="W20" t="s">
-        <v>19</v>
+        <v>0.0007831034</v>
+      </c>
+      <c r="W20" s="1">
+        <v>0.0002734165</v>
+      </c>
+      <c r="X20" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C21">
-        <v>0.95913800000000005</v>
+        <v>0.959138</v>
       </c>
       <c r="D21">
-        <v>1.0983799999999999</v>
+        <v>1.09838</v>
       </c>
       <c r="E21">
         <v>1.24343</v>
       </c>
       <c r="F21">
-        <v>1.3521300000000001</v>
+        <v>1.35213</v>
       </c>
       <c r="G21">
-        <v>1.4521299999999999</v>
+        <v>1.35213</v>
       </c>
       <c r="H21">
+        <v>1.45213</v>
+      </c>
+      <c r="I21">
         <v>1.55019</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>1.649</v>
       </c>
-      <c r="J21">
-        <v>1.7408699999999999</v>
-      </c>
       <c r="K21">
+        <v>1.74087</v>
+      </c>
+      <c r="L21">
         <v>1.8347</v>
       </c>
-      <c r="L21">
-        <v>1.9335100000000001</v>
-      </c>
       <c r="M21">
+        <v>1.93351</v>
+      </c>
+      <c r="N21">
         <v>2.01763</v>
       </c>
-      <c r="N21">
-        <v>2.0780400000000001</v>
-      </c>
       <c r="O21">
-        <v>2.1179399999999999</v>
+        <v>2.07804</v>
       </c>
       <c r="P21">
-        <v>2.1430199999999999</v>
+        <v>2.11794</v>
       </c>
       <c r="Q21">
-        <v>2.1652999999999998</v>
+        <v>2.14302</v>
       </c>
       <c r="R21">
+        <v>2.1653</v>
+      </c>
+      <c r="S21">
         <v>2.15909</v>
       </c>
-      <c r="S21">
-        <v>2.1387399999999999</v>
-      </c>
       <c r="T21">
-        <v>2.1105700000000001</v>
+        <v>2.13874</v>
       </c>
       <c r="U21">
+        <v>2.11057</v>
+      </c>
+      <c r="V21">
         <v>2.07456</v>
       </c>
-      <c r="V21">
-        <v>2.0306000000000002</v>
-      </c>
-      <c r="W21" t="s">
-        <v>20</v>
+      <c r="W21">
+        <v>2.0306</v>
+      </c>
+      <c r="X21" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24">
       <c r="A22" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C22">
-        <v>2.1581000000000001</v>
+        <v>2.1581</v>
       </c>
       <c r="D22">
-        <v>2.3890899999999999</v>
+        <v>2.38909</v>
       </c>
       <c r="E22">
-        <v>2.6120299999999999</v>
+        <v>2.61203</v>
       </c>
       <c r="F22">
         <v>2.79257</v>
       </c>
       <c r="G22">
+        <v>2.79257</v>
+      </c>
+      <c r="H22">
         <v>2.96332</v>
       </c>
-      <c r="H22">
-        <v>3.1041300000000001</v>
-      </c>
       <c r="I22">
+        <v>3.10413</v>
+      </c>
+      <c r="J22">
         <v>3.21489</v>
       </c>
-      <c r="J22">
-        <v>3.2875399999999999</v>
-      </c>
       <c r="K22">
-        <v>3.3264399999999998</v>
+        <v>3.28754</v>
       </c>
       <c r="L22">
+        <v>3.32644</v>
+      </c>
+      <c r="M22">
         <v>3.34396</v>
       </c>
-      <c r="M22">
-        <v>3.3403299999999998</v>
-      </c>
       <c r="N22">
-        <v>3.3126899999999999</v>
+        <v>3.34033</v>
       </c>
       <c r="O22">
-        <v>3.2643800000000001</v>
+        <v>3.31269</v>
       </c>
       <c r="P22">
-        <v>3.2016399999999998</v>
+        <v>3.26438</v>
       </c>
       <c r="Q22">
-        <v>3.1350600000000002</v>
+        <v>3.20164</v>
       </c>
       <c r="R22">
-        <v>3.0393599999999998</v>
+        <v>3.13506</v>
       </c>
       <c r="S22">
-        <v>2.9274300000000002</v>
+        <v>3.03936</v>
       </c>
       <c r="T22">
-        <v>2.8149899999999999</v>
+        <v>2.92743</v>
       </c>
       <c r="U22">
+        <v>2.81499</v>
+      </c>
+      <c r="V22">
         <v>2.71211</v>
       </c>
-      <c r="V22">
-        <v>2.6254200000000001</v>
-      </c>
-      <c r="W22" t="s">
+      <c r="W22">
+        <v>2.62542</v>
+      </c>
+      <c r="X22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24">
+      <c r="A23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>9</v>
-      </c>
       <c r="B23" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2040,66 +2679,69 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>4.5325749999999996</v>
+        <v>4.532575</v>
       </c>
       <c r="G23">
-        <v>34.857222200000002</v>
+        <v>4.532575</v>
       </c>
       <c r="H23">
-        <v>69.819775199999995</v>
+        <v>34.8572222</v>
       </c>
       <c r="I23">
-        <v>94.444886299999993</v>
+        <v>69.8197752</v>
       </c>
       <c r="J23">
+        <v>94.4448863</v>
+      </c>
+      <c r="K23">
         <v>116.2670339</v>
       </c>
-      <c r="K23">
+      <c r="L23">
         <v>135.2506147</v>
       </c>
-      <c r="L23">
-        <v>156.55535610000001</v>
-      </c>
       <c r="M23">
+        <v>156.5553561</v>
+      </c>
+      <c r="N23">
         <v>203.8154835</v>
       </c>
-      <c r="N23">
-        <v>274.50731230000002</v>
-      </c>
       <c r="O23">
-        <v>367.27883589999999</v>
+        <v>274.5073123</v>
       </c>
       <c r="P23">
-        <v>466.85848120000003</v>
+        <v>367.2788359</v>
       </c>
       <c r="Q23">
-        <v>542.89730259999999</v>
+        <v>466.8584812</v>
       </c>
       <c r="R23">
-        <v>824.86284650000005</v>
+        <v>542.8973026</v>
       </c>
       <c r="S23">
-        <v>1339.5501856000001</v>
+        <v>824.8628465</v>
       </c>
       <c r="T23">
+        <v>1339.5501856</v>
+      </c>
+      <c r="U23">
         <v>1317.1616193</v>
       </c>
-      <c r="U23">
+      <c r="V23">
         <v>1334.2744</v>
       </c>
-      <c r="V23">
+      <c r="W23">
         <v>1393.4177605</v>
       </c>
-      <c r="W23" t="s">
+      <c r="X23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24">
+      <c r="A24" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>16</v>
-      </c>
       <c r="B24" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C24">
         <v>42369.98</v>
@@ -2114,134 +2756,140 @@
         <v>54375.06</v>
       </c>
       <c r="G24">
+        <v>54375.06</v>
+      </c>
+      <c r="H24">
         <v>57890.3</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>61306.98</v>
       </c>
-      <c r="I24">
+      <c r="J24">
         <v>64229.66</v>
       </c>
-      <c r="J24">
+      <c r="K24">
         <v>66435.56</v>
       </c>
-      <c r="K24">
+      <c r="L24">
         <v>67996.66</v>
       </c>
-      <c r="L24">
+      <c r="M24">
         <v>69738.12</v>
       </c>
-      <c r="M24">
-        <v>72269.600000000006</v>
-      </c>
       <c r="N24">
-        <v>74537.210000000006</v>
+        <v>72269.6</v>
       </c>
       <c r="O24">
+        <v>74537.21</v>
+      </c>
+      <c r="P24">
         <v>76573.58</v>
       </c>
-      <c r="P24">
-        <v>78701.570000000007</v>
-      </c>
       <c r="Q24">
+        <v>78701.57</v>
+      </c>
+      <c r="R24">
         <v>79457.59</v>
       </c>
-      <c r="R24">
-        <v>80615.710000000006</v>
-      </c>
       <c r="S24">
+        <v>80615.71</v>
+      </c>
+      <c r="T24">
         <v>81671.41</v>
       </c>
-      <c r="T24">
-        <v>82925.289999999994</v>
-      </c>
       <c r="U24">
+        <v>82925.29</v>
+      </c>
+      <c r="V24">
         <v>84049.22</v>
       </c>
-      <c r="V24">
+      <c r="W24">
         <v>84702.95</v>
       </c>
-      <c r="W24" t="s">
-        <v>17</v>
+      <c r="X24" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24">
       <c r="A25" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C25">
-        <v>8406.4110000000001</v>
+        <v>8406.411</v>
       </c>
       <c r="D25">
         <v>10678.654</v>
       </c>
       <c r="E25">
-        <v>11973.887000000001</v>
+        <v>11973.887</v>
       </c>
       <c r="F25">
         <v>12912.22</v>
       </c>
       <c r="G25">
-        <v>13621.728999999999</v>
+        <v>12912.22</v>
       </c>
       <c r="H25">
-        <v>14085.558999999999</v>
+        <v>13621.729</v>
       </c>
       <c r="I25">
+        <v>14085.559</v>
+      </c>
+      <c r="J25">
         <v>14320.822</v>
       </c>
-      <c r="J25">
+      <c r="K25">
         <v>14506.706</v>
       </c>
-      <c r="K25">
-        <v>14295.074000000001</v>
-      </c>
       <c r="L25">
-        <v>14092.218999999999</v>
+        <v>14295.074</v>
       </c>
       <c r="M25">
-        <v>13843.138999999999</v>
+        <v>14092.219</v>
       </c>
       <c r="N25">
+        <v>13843.139</v>
+      </c>
+      <c r="O25">
         <v>13644.358</v>
       </c>
-      <c r="O25">
-        <v>13330.825999999999</v>
-      </c>
       <c r="P25">
-        <v>12986.620999999999</v>
+        <v>13330.826</v>
       </c>
       <c r="Q25">
+        <v>12986.621</v>
+      </c>
+      <c r="R25">
         <v>12208.233</v>
       </c>
-      <c r="R25">
-        <v>11749.255999999999</v>
-      </c>
       <c r="S25">
+        <v>11749.256</v>
+      </c>
+      <c r="T25">
         <v>11250.071</v>
       </c>
-      <c r="T25">
+      <c r="U25">
         <v>10834.24</v>
       </c>
-      <c r="U25">
+      <c r="V25">
         <v>10426.029</v>
       </c>
-      <c r="V25">
-        <v>9955.2330000000002</v>
-      </c>
-      <c r="W25" t="s">
-        <v>17</v>
+      <c r="W25">
+        <v>9955.233</v>
+      </c>
+      <c r="X25" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24">
       <c r="A26" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B26" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C26">
         <v>30561.83</v>
@@ -2256,63 +2904,66 @@
         <v>39086.61</v>
       </c>
       <c r="G26">
+        <v>39086.61</v>
+      </c>
+      <c r="H26">
         <v>41853.46</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>44077.47</v>
       </c>
-      <c r="I26">
+      <c r="J26">
         <v>46300.61</v>
       </c>
-      <c r="J26">
+      <c r="K26">
         <v>47733.51</v>
       </c>
-      <c r="K26">
+      <c r="L26">
         <v>48653.52</v>
       </c>
-      <c r="L26">
+      <c r="M26">
         <v>49655.56</v>
       </c>
-      <c r="M26">
+      <c r="N26">
         <v>51370.65</v>
       </c>
-      <c r="N26">
-        <v>52964.480000000003</v>
-      </c>
       <c r="O26">
+        <v>52964.48</v>
+      </c>
+      <c r="P26">
         <v>54384.73</v>
       </c>
-      <c r="P26">
+      <c r="Q26">
         <v>55845.68</v>
       </c>
-      <c r="Q26">
+      <c r="R26">
         <v>56058.61</v>
       </c>
-      <c r="R26">
+      <c r="S26">
         <v>56691.95</v>
       </c>
-      <c r="S26">
+      <c r="T26">
         <v>57175.7</v>
       </c>
-      <c r="T26">
+      <c r="U26">
         <v>57909.17</v>
       </c>
-      <c r="U26">
+      <c r="V26">
         <v>59306.3</v>
       </c>
-      <c r="V26">
+      <c r="W26">
         <v>59486.45</v>
       </c>
-      <c r="W26" t="s">
-        <v>18</v>
+      <c r="X26" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:24">
       <c r="A27" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B27" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C27">
         <v>29385.9</v>
@@ -2327,69 +2978,72 @@
         <v>40748.65</v>
       </c>
       <c r="G27">
+        <v>40748.65</v>
+      </c>
+      <c r="H27">
         <v>43323.08</v>
       </c>
-      <c r="H27">
+      <c r="I27">
         <v>45098.89</v>
       </c>
-      <c r="I27">
+      <c r="J27">
         <v>46560.36</v>
       </c>
-      <c r="J27">
+      <c r="K27">
         <v>48060.11</v>
       </c>
-      <c r="K27">
+      <c r="L27">
         <v>49156.74</v>
       </c>
-      <c r="L27">
+      <c r="M27">
         <v>50316.07</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>51822.65</v>
       </c>
-      <c r="N27">
+      <c r="O27">
         <v>53305.49</v>
       </c>
-      <c r="O27">
+      <c r="P27">
         <v>54755.48</v>
       </c>
-      <c r="P27">
-        <v>56098.080000000002</v>
-      </c>
       <c r="Q27">
+        <v>56098.08</v>
+      </c>
+      <c r="R27">
         <v>56358.68</v>
       </c>
-      <c r="R27">
+      <c r="S27">
         <v>56981.99</v>
       </c>
-      <c r="S27">
+      <c r="T27">
         <v>57457.09</v>
       </c>
-      <c r="T27">
+      <c r="U27">
         <v>58140.31</v>
       </c>
-      <c r="U27">
+      <c r="V27">
         <v>59538.46</v>
       </c>
-      <c r="V27">
+      <c r="W27">
         <v>59655.22</v>
       </c>
-      <c r="W27" t="s">
-        <v>18</v>
+      <c r="X27" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:24">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B28" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C28">
         <v>6531.71</v>
       </c>
       <c r="D28">
-        <v>8494.4169999999995</v>
+        <v>8494.417</v>
       </c>
       <c r="E28">
         <v>10052.304</v>
@@ -2398,69 +3052,72 @@
         <v>10929.632</v>
       </c>
       <c r="G28">
+        <v>10929.632</v>
+      </c>
+      <c r="H28">
         <v>11612.525</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>12061.752</v>
       </c>
-      <c r="I28">
-        <v>12284.656000000001</v>
-      </c>
       <c r="J28">
+        <v>12284.656</v>
+      </c>
+      <c r="K28">
         <v>12446.279</v>
       </c>
-      <c r="K28">
+      <c r="L28">
         <v>12231.152</v>
       </c>
-      <c r="L28">
+      <c r="M28">
         <v>12028.258</v>
       </c>
-      <c r="M28">
+      <c r="N28">
         <v>11768.822</v>
       </c>
-      <c r="N28">
-        <v>11562.102000000001</v>
-      </c>
       <c r="O28">
+        <v>11562.102</v>
+      </c>
+      <c r="P28">
         <v>11250.186</v>
       </c>
-      <c r="P28">
-        <v>10908.914000000001</v>
-      </c>
       <c r="Q28">
-        <v>10163.449000000001</v>
+        <v>10908.914</v>
       </c>
       <c r="R28">
-        <v>9727.6810000000005</v>
+        <v>10163.449</v>
       </c>
       <c r="S28">
-        <v>9242.8160000000007</v>
+        <v>9727.681</v>
       </c>
       <c r="T28">
-        <v>8864.6650000000009</v>
+        <v>9242.816</v>
       </c>
       <c r="U28">
-        <v>8488.9779999999992</v>
+        <v>8864.665</v>
       </c>
       <c r="V28">
-        <v>8066.2240000000002</v>
-      </c>
-      <c r="W28" t="s">
-        <v>18</v>
+        <v>8488.978</v>
+      </c>
+      <c r="W28">
+        <v>8066.224</v>
+      </c>
+      <c r="X28" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24">
       <c r="A29" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B29" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C29">
         <v>6471.384</v>
       </c>
       <c r="D29">
-        <v>8745.7739999999994</v>
+        <v>8745.774</v>
       </c>
       <c r="E29">
         <v>10353.989</v>
@@ -2469,351 +3126,367 @@
         <v>11178.46</v>
       </c>
       <c r="G29">
+        <v>11178.46</v>
+      </c>
+      <c r="H29">
         <v>11834.778</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>12261.919</v>
       </c>
-      <c r="I29">
-        <v>12446.619000000001</v>
-      </c>
       <c r="J29">
+        <v>12446.619</v>
+      </c>
+      <c r="K29">
         <v>12586.036</v>
       </c>
-      <c r="K29">
+      <c r="L29">
         <v>12368.591</v>
       </c>
-      <c r="L29">
+      <c r="M29">
         <v>12174.526</v>
       </c>
-      <c r="M29">
-        <v>11889.994000000001</v>
-      </c>
       <c r="N29">
+        <v>11889.994</v>
+      </c>
+      <c r="O29">
         <v>11664.953</v>
       </c>
-      <c r="O29">
+      <c r="P29">
         <v>11342.796</v>
       </c>
-      <c r="P29">
-        <v>10990.406999999999</v>
-      </c>
       <c r="Q29">
-        <v>10242.264999999999</v>
+        <v>10990.407</v>
       </c>
       <c r="R29">
-        <v>9804.7139999999999</v>
+        <v>10242.265</v>
       </c>
       <c r="S29">
-        <v>9319.6200000000008</v>
+        <v>9804.714</v>
       </c>
       <c r="T29">
-        <v>8938.9210000000003</v>
+        <v>9319.62</v>
       </c>
       <c r="U29">
-        <v>8558.6869999999999</v>
+        <v>8938.921</v>
       </c>
       <c r="V29">
-        <v>8119.8879999999999</v>
-      </c>
-      <c r="W29" t="s">
-        <v>18</v>
+        <v>8558.687</v>
+      </c>
+      <c r="W29">
+        <v>8119.888</v>
+      </c>
+      <c r="X29" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24">
       <c r="A30" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B30" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C30">
-        <v>2541.1350000000002</v>
+        <v>2541.135</v>
       </c>
       <c r="D30">
-        <v>4246.8239999999996</v>
+        <v>4246.824</v>
       </c>
       <c r="E30">
         <v>5443.79</v>
       </c>
       <c r="F30">
-        <v>6593.1480000000001</v>
+        <v>6593.148</v>
       </c>
       <c r="G30">
-        <v>7831.4040000000005</v>
+        <v>6593.148</v>
       </c>
       <c r="H30">
-        <v>8520.4860000000008</v>
+        <v>7831.404</v>
       </c>
       <c r="I30">
-        <v>8899.6959999999999</v>
+        <v>8520.486</v>
       </c>
       <c r="J30">
-        <v>9527.1350000000002</v>
+        <v>8899.696</v>
       </c>
       <c r="K30">
-        <v>9862.4590000000007</v>
+        <v>9527.135</v>
       </c>
       <c r="L30">
-        <v>10333.004999999999</v>
+        <v>9862.459</v>
       </c>
       <c r="M30">
+        <v>10333.005</v>
+      </c>
+      <c r="N30">
         <v>10469.989</v>
       </c>
-      <c r="N30">
+      <c r="O30">
         <v>10563.196</v>
       </c>
-      <c r="O30">
-        <v>10414.906000000001</v>
-      </c>
       <c r="P30">
+        <v>10414.906</v>
+      </c>
+      <c r="Q30">
         <v>10273.288</v>
       </c>
-      <c r="Q30">
-        <v>9938.0400000000009</v>
-      </c>
       <c r="R30">
-        <v>9654.0190000000002</v>
+        <v>9938.04</v>
       </c>
       <c r="S30">
-        <v>9424.7890000000007</v>
+        <v>9654.019</v>
       </c>
       <c r="T30">
+        <v>9424.789</v>
+      </c>
+      <c r="U30">
         <v>9156.134</v>
       </c>
-      <c r="U30">
-        <v>8782.3649999999998</v>
-      </c>
       <c r="V30">
-        <v>8519.5920000000006</v>
-      </c>
-      <c r="W30" t="s">
-        <v>19</v>
+        <v>8782.365</v>
+      </c>
+      <c r="W30">
+        <v>8519.592</v>
+      </c>
+      <c r="X30" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24">
       <c r="A31" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B31" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C31" s="1">
         <v>2001.721</v>
       </c>
       <c r="D31" s="1">
-        <v>3296.4760000000001</v>
+        <v>3296.476</v>
       </c>
       <c r="E31" s="1">
-        <v>3996.4389999999999</v>
+        <v>3996.439</v>
       </c>
       <c r="F31" s="1">
-        <v>4368.5039999999999</v>
+        <v>4368.504</v>
       </c>
       <c r="G31" s="1">
+        <v>4368.504</v>
+      </c>
+      <c r="H31" s="1">
         <v>4710.34</v>
       </c>
-      <c r="H31" s="1">
-        <v>4592.2129999999997</v>
-      </c>
       <c r="I31" s="1">
-        <v>4674.9489999999996</v>
+        <v>4592.213</v>
       </c>
       <c r="J31" s="1">
-        <v>4807.5929999999998</v>
+        <v>4674.949</v>
       </c>
       <c r="K31" s="1">
+        <v>4807.593</v>
+      </c>
+      <c r="L31" s="1">
         <v>4770.17</v>
       </c>
-      <c r="L31" s="1">
-        <v>4829.2820000000002</v>
-      </c>
       <c r="M31" s="1">
-        <v>4864.8190000000004</v>
+        <v>4829.282</v>
       </c>
       <c r="N31" s="1">
-        <v>4919.2030000000004</v>
+        <v>4864.819</v>
       </c>
       <c r="O31" s="1">
+        <v>4919.203</v>
+      </c>
+      <c r="P31" s="1">
         <v>4855.59</v>
       </c>
-      <c r="P31" s="1">
-        <v>4803.4359999999997</v>
-      </c>
       <c r="Q31" s="1">
-        <v>4353.7759999999998</v>
+        <v>4803.436</v>
       </c>
       <c r="R31" s="1">
+        <v>4353.776</v>
+      </c>
+      <c r="S31" s="1">
         <v>4210.884</v>
       </c>
-      <c r="S31" s="1">
-        <v>4050.9349999999999</v>
-      </c>
       <c r="T31" s="1">
-        <v>3952.6060000000002</v>
+        <v>4050.935</v>
       </c>
       <c r="U31" s="1">
+        <v>3952.606</v>
+      </c>
+      <c r="V31" s="1">
         <v>3708.585</v>
       </c>
-      <c r="V31" s="1">
+      <c r="W31" s="1">
         <v>3504.51</v>
       </c>
-      <c r="W31" t="s">
-        <v>19</v>
+      <c r="X31" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C32">
-        <v>0.95913800000000005</v>
+        <v>0.959138</v>
       </c>
       <c r="D32">
-        <v>1.0983799999999999</v>
+        <v>1.09838</v>
       </c>
       <c r="E32">
         <v>1.24343</v>
       </c>
       <c r="F32">
-        <v>1.3646400000000001</v>
+        <v>1.36464</v>
       </c>
       <c r="G32">
-        <v>1.4885999999999999</v>
+        <v>1.36464</v>
       </c>
       <c r="H32">
+        <v>1.4886</v>
+      </c>
+      <c r="I32">
         <v>1.61372</v>
       </c>
-      <c r="I32">
+      <c r="J32">
         <v>1.73777</v>
       </c>
-      <c r="J32">
+      <c r="K32">
         <v>1.85717</v>
       </c>
-      <c r="K32">
+      <c r="L32">
         <v>1.97824</v>
       </c>
-      <c r="L32">
-        <v>2.1154000000000002</v>
-      </c>
       <c r="M32">
-        <v>2.2639300000000002</v>
+        <v>2.1154</v>
       </c>
       <c r="N32">
-        <v>2.4270100000000001</v>
+        <v>2.26393</v>
       </c>
       <c r="O32">
-        <v>2.5968100000000001</v>
+        <v>2.42701</v>
       </c>
       <c r="P32">
-        <v>2.7700999999999998</v>
+        <v>2.59681</v>
       </c>
       <c r="Q32">
-        <v>2.9524900000000001</v>
+        <v>2.7701</v>
       </c>
       <c r="R32">
-        <v>3.1354500000000001</v>
+        <v>2.95249</v>
       </c>
       <c r="S32">
+        <v>3.13545</v>
+      </c>
+      <c r="T32">
         <v>3.32016</v>
       </c>
-      <c r="T32">
-        <v>3.5057200000000002</v>
-      </c>
       <c r="U32">
-        <v>3.6870599999999998</v>
+        <v>3.50572</v>
       </c>
       <c r="V32">
-        <v>3.8634400000000002</v>
-      </c>
-      <c r="W32" t="s">
-        <v>20</v>
+        <v>3.68706</v>
+      </c>
+      <c r="W32">
+        <v>3.86344</v>
+      </c>
+      <c r="X32" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:24">
       <c r="A33" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B33" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C33">
-        <v>2.1581000000000001</v>
+        <v>2.1581</v>
       </c>
       <c r="D33">
-        <v>2.3890899999999999</v>
+        <v>2.38909</v>
       </c>
       <c r="E33">
-        <v>2.6120299999999999</v>
+        <v>2.61203</v>
       </c>
       <c r="F33">
         <v>2.81528</v>
       </c>
       <c r="G33">
-        <v>3.0405799999999998</v>
+        <v>2.81528</v>
       </c>
       <c r="H33">
-        <v>3.2748200000000001</v>
+        <v>3.04058</v>
       </c>
       <c r="I33">
-        <v>3.5067200000000001</v>
+        <v>3.27482</v>
       </c>
       <c r="J33">
+        <v>3.50672</v>
+      </c>
+      <c r="K33">
         <v>3.72715</v>
       </c>
-      <c r="K33">
-        <v>3.9306899999999998</v>
-      </c>
       <c r="L33">
-        <v>4.1290399999999998</v>
+        <v>3.93069</v>
       </c>
       <c r="M33">
-        <v>4.3294300000000003</v>
+        <v>4.12904</v>
       </c>
       <c r="N33">
-        <v>4.5426900000000003</v>
+        <v>4.32943</v>
       </c>
       <c r="O33">
+        <v>4.54269</v>
+      </c>
+      <c r="P33">
         <v>4.76152</v>
       </c>
-      <c r="P33">
-        <v>4.9847999999999999</v>
-      </c>
       <c r="Q33">
-        <v>5.2172999999999998</v>
+        <v>4.9848</v>
       </c>
       <c r="R33">
-        <v>5.4436499999999999</v>
+        <v>5.2173</v>
       </c>
       <c r="S33">
-        <v>5.6655600000000002</v>
+        <v>5.44365</v>
       </c>
       <c r="T33">
-        <v>5.8832199999999997</v>
+        <v>5.66556</v>
       </c>
       <c r="U33">
-        <v>6.0937299999999999</v>
+        <v>5.88322</v>
       </c>
       <c r="V33">
-        <v>6.2992299999999997</v>
-      </c>
-      <c r="W33" t="s">
-        <v>21</v>
+        <v>6.09373</v>
+      </c>
+      <c r="W33">
+        <v>6.29923</v>
+      </c>
+      <c r="X33" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B34" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>